<commit_message>
Edit Code RegisterStudent, Login, LoginAdmin, DepositMoney, AddCourse, RegisterCourse
</commit_message>
<xml_diff>
--- a/ExcelProject/Deposit_Money.xlsx
+++ b/ExcelProject/Deposit_Money.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="24">
   <si>
     <t>Execute</t>
   </si>
@@ -46,28 +46,40 @@
     <t>เติมเงินสำเร็จ</t>
   </si>
   <si>
+    <t>เงินฝากสำเร็จแล้ว จำนวน: 101 บาท กด OK เพื่อกลับหน้า Home</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
     <t>TC7:02</t>
   </si>
   <si>
     <t>กรุณากรอกเป็นตัวเลขจำนวนเต็มเป็นเงินบาท</t>
   </si>
   <si>
+    <t>เงินฝากสำเร็จแล้ว จำนวน: 1000 บาท กด OK เพื่อกลับหน้า Home</t>
+  </si>
+  <si>
     <t>TC7:03</t>
   </si>
   <si>
     <t>TC7:04</t>
   </si>
   <si>
+    <t>เงินฝากสำเร็จแล้ว จำนวน: 100 บาท กด OK เพื่อกลับหน้า Home</t>
+  </si>
+  <si>
+    <t>TC7:05</t>
+  </si>
+  <si>
+    <t>จำนวนเงินขั้นต่ำคือ 100 บาท</t>
+  </si>
+  <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>TC7:05</t>
-  </si>
-  <si>
-    <t>ยอดเงินขั้นต่ำ 100 บาท</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>TC7:06</t>
@@ -80,7 +92,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -160,12 +174,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -174,34 +188,25 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -509,13 +514,13 @@
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="13" width="9.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="13" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="9.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="13" width="27.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="13" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="13" width="26.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="9.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="11" width="9.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="27.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="41.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="10" width="26.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="27">
@@ -541,7 +546,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -554,33 +559,45 @@
       <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
+      <c r="E2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="5">
+        <v>13</v>
+      </c>
+      <c r="C3" s="6">
         <v>100.5</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
+      <c r="G3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C4" s="5">
         <v>100</v>
@@ -588,16 +605,22 @@
       <c r="D4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C5" s="5">
         <v>101</v>
@@ -605,88 +628,104 @@
       <c r="D5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
+      <c r="E5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C6" s="5">
         <v>99</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="22.5">
+        <v>20</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
-      <c r="A9" s="11"/>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21">
+      <c r="A9" s="9"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
-      <c r="A10" s="11"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21">
+      <c r="A10" s="9"/>
       <c r="B10" s="8"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
-      <c r="A11" s="11"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21">
+      <c r="A11" s="9"/>
       <c r="B11" s="8"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
-      <c r="A12" s="11"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21">
+      <c r="A12" s="9"/>
       <c r="B12" s="8"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add File Edit 9/11
</commit_message>
<xml_diff>
--- a/ExcelProject/Deposit_Money.xlsx
+++ b/ExcelProject/Deposit_Money.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
   <si>
     <t>Execute</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Revise</t>
   </si>
   <si>
-    <t>N</t>
+    <t>Y</t>
   </si>
   <si>
     <t>TC7:01</t>
@@ -46,40 +46,37 @@
     <t>เติมเงินสำเร็จ</t>
   </si>
   <si>
-    <t>เงินฝากสำเร็จแล้ว จำนวน: 101 บาท กด OK เพื่อกลับหน้า Home</t>
+    <t>เงินฝากสำเร็จแล้ว จำนวน: 500 บาท กด OK เพื่อกลับหน้า Home</t>
   </si>
   <si>
     <t>Fail</t>
   </si>
   <si>
+    <t>TC7:02</t>
+  </si>
+  <si>
+    <t>กรุณากรอกเป็นตัวเลขจำนวนเต็มเป็นเงินบาท</t>
+  </si>
+  <si>
+    <t>เงินฝากสำเร็จแล้ว จำนวน: 1000 บาท กด OK เพื่อกลับหน้า Home</t>
+  </si>
+  <si>
+    <t>TC7:03</t>
+  </si>
+  <si>
+    <t>TC7:04</t>
+  </si>
+  <si>
+    <t>เงินฝากสำเร็จแล้ว จำนวน: 100 บาท กด OK เพื่อกลับหน้า Home</t>
+  </si>
+  <si>
+    <t>TC7:05</t>
+  </si>
+  <si>
+    <t>จำนวนเงินขั้นต่ำคือ 100 บาท</t>
+  </si>
+  <si>
     <t>Pass</t>
-  </si>
-  <si>
-    <t>TC7:02</t>
-  </si>
-  <si>
-    <t>กรุณากรอกเป็นตัวเลขจำนวนเต็มเป็นเงินบาท</t>
-  </si>
-  <si>
-    <t>เงินฝากสำเร็จแล้ว จำนวน: 1000 บาท กด OK เพื่อกลับหน้า Home</t>
-  </si>
-  <si>
-    <t>TC7:03</t>
-  </si>
-  <si>
-    <t>TC7:04</t>
-  </si>
-  <si>
-    <t>เงินฝากสำเร็จแล้ว จำนวน: 100 บาท กด OK เพื่อกลับหน้า Home</t>
-  </si>
-  <si>
-    <t>TC7:05</t>
-  </si>
-  <si>
-    <t>จำนวนเงินขั้นต่ำคือ 100 บาท</t>
-  </si>
-  <si>
-    <t>Y</t>
   </si>
   <si>
     <t>TC7:06</t>
@@ -523,7 +520,7 @@
     <col min="7" max="7" style="10" width="26.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="27">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="27.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -566,7 +563,7 @@
         <v>11</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21">
@@ -574,16 +571,16 @@
         <v>7</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="6">
         <v>100.5</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>11</v>
@@ -597,7 +594,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="5">
         <v>100</v>
@@ -606,13 +603,13 @@
         <v>9</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21">
@@ -620,7 +617,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="5">
         <v>101</v>
@@ -629,13 +626,13 @@
         <v>9</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21">
@@ -643,43 +640,43 @@
         <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="5">
         <v>99</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
       <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>22</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">

</xml_diff>